<commit_message>
plots and optgp sampling updates
</commit_message>
<xml_diff>
--- a/smoment/autopacmen_output/Mitocore_aligned_to_Human1/Mitocore_aligned_to_Human1_kcats_calibrated.xlsx
+++ b/smoment/autopacmen_output/Mitocore_aligned_to_Human1/Mitocore_aligned_to_Human1_kcats_calibrated.xlsx
@@ -1,15 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emanuel.lange\git\mitocore-smoment-model\smoment\autopacmen_output\Mitocore_aligned_to_Human1\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C19B543A-BE58-42F7-AB69-B265BB68BBB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
@@ -73,8 +79,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -133,17 +139,25 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -181,7 +195,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -215,6 +229,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -249,9 +264,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -424,11 +440,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C16"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="19.453125" customWidth="1"/>
+    <col min="2" max="2" width="21.26953125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -439,7 +459,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -447,10 +467,10 @@
         <v>18.5</v>
       </c>
       <c r="C2">
-        <v>340.2551854062008</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
+        <v>340.25518540620078</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -458,10 +478,10 @@
         <v>79</v>
       </c>
       <c r="C3">
-        <v>3950.402820655703</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
+        <v>3950.4028206557032</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
@@ -469,10 +489,10 @@
         <v>38.1</v>
       </c>
       <c r="C4">
-        <v>1905.19839147501</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
+        <v>1905.1983914750101</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
@@ -480,10 +500,10 @@
         <v>13.33333</v>
       </c>
       <c r="C5">
-        <v>666.7359283203543</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
+        <v>666.73592832035433</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>7</v>
       </c>
@@ -494,7 +514,7 @@
         <v>1597.414479786109</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>8</v>
       </c>
@@ -505,7 +525,7 @@
         <v>1597.414479786109</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>9</v>
       </c>
@@ -513,21 +533,21 @@
         <v>5.2</v>
       </c>
       <c r="C8">
-        <v>260.0280421193248</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3">
+        <v>260.02804211932482</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B9">
-        <v>12.03333</v>
+        <v>12.033329999999999</v>
       </c>
       <c r="C9">
-        <v>601.7361139186795</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3">
+        <v>601.73611391867951</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>11</v>
       </c>
@@ -535,10 +555,10 @@
         <v>3.5</v>
       </c>
       <c r="C10">
-        <v>175.0202478212912</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3">
+        <v>175.02024782129121</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>12</v>
       </c>
@@ -549,18 +569,18 @@
         <v>260.0268909903491</v>
       </c>
     </row>
-    <row r="12" spans="1:3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B12">
-        <v>0.57</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="C12">
-        <v>28.50287978266452</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3">
+        <v>28.502879782664522</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>14</v>
       </c>
@@ -568,10 +588,10 @@
         <v>19.8</v>
       </c>
       <c r="C13">
-        <v>990.0937079405626</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3">
+        <v>990.09370794056258</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>15</v>
       </c>
@@ -579,10 +599,10 @@
         <v>27.15</v>
       </c>
       <c r="C14">
-        <v>1357.628219520483</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3">
+        <v>1357.6282195204831</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>16</v>
       </c>
@@ -590,18 +610,18 @@
         <v>27.15</v>
       </c>
       <c r="C15">
-        <v>1357.628219520483</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3">
+        <v>1357.6282195204831</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B16">
-        <v>0.57</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="C16">
-        <v>28.50337196632104</v>
+        <v>28.503371966321041</v>
       </c>
     </row>
   </sheetData>

</xml_diff>